<commit_message>
Update range and charging anxiety cost assumptions
</commit_message>
<xml_diff>
--- a/InputData/trans/BNoGP/BAU Number of Gas Pumps.xlsx
+++ b/InputData/trans/BNoGP/BAU Number of Gas Pumps.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mdeng\Desktop\Dropbox_Free_Zone\EPS\Model Repos\eps-us\InputData\trans\BNoGP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\trans\BNoGP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D1B5AEA-3A11-463F-9E0D-2C706DCF7B19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D8385F-0EDF-4884-99C4-2E50D11FE4CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="555" yWindow="885" windowWidth="22950" windowHeight="13650" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Source:</t>
   </si>
@@ -51,25 +51,28 @@
     <t>Number of Gas pumps</t>
   </si>
   <si>
-    <t>CleanTechnica</t>
-  </si>
-  <si>
-    <t>Stop Comparing the Number of Gas Stations to EV Charging Stations</t>
-  </si>
-  <si>
-    <t>https://cleantechnica.com/2018/03/07/stop-comparing-number-gas-stations-ev-charging-stations/</t>
-  </si>
-  <si>
     <t>Number of chargers</t>
   </si>
   <si>
-    <t>We assume the number of gas pumps remains relatively constant.</t>
-  </si>
-  <si>
     <t>BNoEVC BAU Number of Gas Pumps</t>
   </si>
   <si>
     <t>BAU Gas Pumps</t>
+  </si>
+  <si>
+    <t>https://www.xmap.ai/blog/gas-stations-in-united-states-of-america-everything-you-need-to-know</t>
+  </si>
+  <si>
+    <t>Gas stations in the United States of America</t>
+  </si>
+  <si>
+    <t>Xmap</t>
+  </si>
+  <si>
+    <t>We assume the number of gas stations remains relatively constant.</t>
+  </si>
+  <si>
+    <t>We assume an average of 8 pumps per gas station.</t>
   </si>
 </sst>
 </file>
@@ -419,19 +422,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" customWidth="1"/>
-    <col min="2" max="2" width="31.85546875" customWidth="1"/>
+    <col min="1" max="1" width="16.54296875" customWidth="1"/>
+    <col min="2" max="2" width="31.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -439,34 +442,39 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B5" s="5">
-        <v>2018</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>7</v>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -480,202 +488,211 @@
   <sheetPr>
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AC2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1">
-        <v>2021</v>
-      </c>
-      <c r="C1" s="3">
-        <v>2022</v>
-      </c>
-      <c r="D1">
-        <v>2023</v>
-      </c>
-      <c r="E1" s="3">
+        <v>3</v>
+      </c>
+      <c r="B1" s="3">
         <v>2024</v>
       </c>
-      <c r="F1">
+      <c r="C1">
         <v>2025</v>
       </c>
-      <c r="G1" s="3">
+      <c r="D1" s="3">
         <v>2026</v>
       </c>
-      <c r="H1">
+      <c r="E1">
         <v>2027</v>
       </c>
-      <c r="I1" s="3">
+      <c r="F1" s="3">
         <v>2028</v>
       </c>
-      <c r="J1">
+      <c r="G1">
         <v>2029</v>
       </c>
-      <c r="K1" s="3">
+      <c r="H1" s="3">
         <v>2030</v>
       </c>
-      <c r="L1">
+      <c r="I1">
         <v>2031</v>
       </c>
-      <c r="M1" s="3">
+      <c r="J1" s="3">
         <v>2032</v>
       </c>
-      <c r="N1">
+      <c r="K1">
         <v>2033</v>
       </c>
-      <c r="O1" s="3">
+      <c r="L1" s="3">
         <v>2034</v>
       </c>
-      <c r="P1">
+      <c r="M1">
         <v>2035</v>
       </c>
-      <c r="Q1" s="3">
+      <c r="N1" s="3">
         <v>2036</v>
       </c>
-      <c r="R1">
+      <c r="O1">
         <v>2037</v>
       </c>
-      <c r="S1" s="3">
+      <c r="P1" s="3">
         <v>2038</v>
       </c>
-      <c r="T1">
+      <c r="Q1">
         <v>2039</v>
       </c>
-      <c r="U1" s="3">
+      <c r="R1" s="3">
         <v>2040</v>
       </c>
-      <c r="V1">
+      <c r="S1">
         <v>2041</v>
       </c>
-      <c r="W1" s="3">
+      <c r="T1" s="3">
         <v>2042</v>
       </c>
-      <c r="X1">
+      <c r="U1">
         <v>2043</v>
       </c>
-      <c r="Y1" s="3">
+      <c r="V1" s="3">
         <v>2044</v>
       </c>
-      <c r="Z1">
+      <c r="W1">
         <v>2045</v>
       </c>
-      <c r="AA1" s="3">
+      <c r="X1" s="3">
         <v>2046</v>
       </c>
-      <c r="AB1">
+      <c r="Y1">
         <v>2047</v>
       </c>
-      <c r="AC1" s="3">
+      <c r="Z1" s="3">
         <v>2048</v>
       </c>
-      <c r="AD1">
+      <c r="AA1">
         <v>2049</v>
       </c>
-      <c r="AE1" s="3">
+      <c r="AB1" s="3">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B2">
-        <v>1200000</v>
+        <f>196643*8</f>
+        <v>1573144</v>
       </c>
       <c r="C2">
-        <v>1200000</v>
+        <f t="shared" ref="C2:AB2" si="0">196643*8</f>
+        <v>1573144</v>
       </c>
       <c r="D2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="E2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="F2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="G2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="H2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="I2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="J2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="K2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="L2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="M2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="N2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="O2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="P2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="Q2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="R2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="S2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="T2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="U2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="V2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="W2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="X2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="Y2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="Z2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="AA2">
-        <v>1200000</v>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
       </c>
       <c r="AB2">
-        <v>1200000</v>
-      </c>
-      <c r="AC2">
-        <v>1200000</v>
-      </c>
-      <c r="AD2">
-        <v>1200000</v>
-      </c>
-      <c r="AE2">
-        <v>1200000</v>
-      </c>
-      <c r="AF2" s="2"/>
+        <f t="shared" si="0"/>
+        <v>1573144</v>
+      </c>
+      <c r="AC2" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>